<commit_message>
Ensuring Duplicates and Bpundary Changes have not disrupted data: COME BACK TO HERE IF NEEDED
</commit_message>
<xml_diff>
--- a/4. output/Table Results.xlsx
+++ b/4. output/Table Results.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stummuac-my.sharepoint.com/personal/25943553_stu_mmu_ac_uk/Documents/03 DISSERTATION/GITHUB/4. output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="206" documentId="11_F25DC773A252ABDACC10484DD11954905ADE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74F55ACC-9FB4-415E-B331-92985E51C5B2}"/>
+  <xr:revisionPtr revIDLastSave="218" documentId="11_F25DC773A252ABDACC10484DD11954905ADE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A963B35E-FE0F-4744-8797-8ADBC1B96040}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="795" windowWidth="19200" windowHeight="9810" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1740" yWindow="180" windowWidth="24300" windowHeight="15375" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Event Studies" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="49">
   <si>
     <t>Outcome</t>
   </si>
@@ -64,9 +64,6 @@
     <t>total_tier</t>
   </si>
   <si>
-    <t>total_retail</t>
-  </si>
-  <si>
     <t>dtp_24m</t>
   </si>
   <si>
@@ -88,9 +85,6 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>Borderline</t>
-  </si>
-  <si>
     <t>Fail</t>
   </si>
   <si>
@@ -139,9 +133,6 @@
     <t>*0.05 **0.001</t>
   </si>
   <si>
-    <t>2014*, 2015*, 2016*, 2018**</t>
-  </si>
-  <si>
     <t>−0.0435 (p&lt;.001)</t>
   </si>
   <si>
@@ -151,36 +142,18 @@
     <t>2021**, 2022**, 2023*, 2024**, 2025**</t>
   </si>
   <si>
-    <t>−0.3211 (p&lt;.001)</t>
-  </si>
-  <si>
-    <t>2020* only</t>
-  </si>
-  <si>
     <t>−0.0278 (p=.001)</t>
   </si>
   <si>
     <t>2014 (p=.042) only</t>
   </si>
   <si>
-    <t>−0.2745 (p&lt;.001)</t>
-  </si>
-  <si>
     <t>None sig.</t>
   </si>
   <si>
-    <t>2022**; borderline 2023 (p=.050), 2025 (p=.050)</t>
-  </si>
-  <si>
     <t>−0.0425 (p=.003)</t>
   </si>
   <si>
-    <t>−0.5207 (p&lt;.001)</t>
-  </si>
-  <si>
-    <t>2020**, 2022*, 2023*</t>
-  </si>
-  <si>
     <t>−0.0296 (p&lt;.001)</t>
   </si>
   <si>
@@ -190,67 +163,28 @@
     <t>2024**, 2025**; borderline 2023 (p=.063)</t>
   </si>
   <si>
-    <t>−0.2471 (p&lt;.001)</t>
-  </si>
-  <si>
-    <t>2014** (strong)</t>
-  </si>
-  <si>
     <t>−0.0704 (p=.002)</t>
   </si>
   <si>
-    <t>−0.8595 (p&lt;.001)</t>
-  </si>
-  <si>
-    <t>2014**, 2015*, 2016*</t>
-  </si>
-  <si>
-    <t>2020*, 2023*, 2024**, 2025**</t>
-  </si>
-  <si>
     <t>−0.0265 (p=.001)</t>
   </si>
   <si>
     <t>2014*, 2015*, 2018*</t>
   </si>
   <si>
-    <t>−0.3006 (p&lt;.001)</t>
-  </si>
-  <si>
-    <t>2018* only</t>
-  </si>
-  <si>
     <t>−0.0657 (p=.002)</t>
   </si>
   <si>
     <t>2014**, 2015*</t>
   </si>
   <si>
-    <t>−0.7344 (p&lt;.001)</t>
-  </si>
-  <si>
-    <t>2020*, 2025* only</t>
-  </si>
-  <si>
-    <t>Pass (borderline)</t>
-  </si>
-  <si>
     <t>2021**–2025** (all sig.)</t>
   </si>
   <si>
     <t>2020*–2025** (all sig.)</t>
   </si>
   <si>
-    <t>2022*–2025** (all sig.)</t>
-  </si>
-  <si>
     <t>2020**–2025** (all sig.)</t>
-  </si>
-  <si>
-    <t>2021*–2025** (all sig.)</t>
-  </si>
-  <si>
-    <t>2016*</t>
   </si>
 </sst>
 </file>
@@ -416,8 +350,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6655E4B7-F89B-4000-BD85-0F21A0B2F9EF}" name="Table1" displayName="Table1" ref="A1:F15" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:F15" xr:uid="{6655E4B7-F89B-4000-BD85-0F21A0B2F9EF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6655E4B7-F89B-4000-BD85-0F21A0B2F9EF}" name="Table1" displayName="Table1" ref="A1:F8" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:F8" xr:uid="{6655E4B7-F89B-4000-BD85-0F21A0B2F9EF}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{DD892928-B6BC-4DDB-9015-DFA0B458F094}" name="Outcome" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{48269CF3-7983-49AE-BAB2-97AC80F00FF9}" name="Variable" dataDxfId="8"/>
@@ -693,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" customWidth="1"/>
@@ -732,35 +666,39 @@
         <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D3" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" s="6"/>
       <c r="E3" s="3" t="s">
-        <v>64</v>
+        <v>14</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
@@ -768,225 +706,99 @@
         <v>7</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="6"/>
       <c r="E5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>36</v>
+      </c>
       <c r="E6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="F7" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F17" t="s">
-        <v>32</v>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F10" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1012,6 +824,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F87F53E-35E7-48A7-BA0D-AEC22765205C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F08F7B5C-6A56-4534-B1CE-5BA013F3959E}">
   <dimension ref="A2:L4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1031,16 +852,16 @@
   <sheetData>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="B2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
@@ -1048,72 +869,72 @@
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="K2" s="7"/>
       <c r="L2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="D3" s="5">
         <v>8</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F3" s="5">
         <v>12</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H3" s="5">
         <v>16</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J3" s="5">
         <v>1</v>
       </c>
       <c r="K3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D4" s="5">
         <v>1</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F4" s="5">
         <v>2</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
@@ -1121,10 +942,10 @@
         <v>2</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>